<commit_message>
feat(PDG-3): map FBI-WANTED source and set date_order
</commit_message>
<xml_diff>
--- a/data/rules/riskClassification.xlsx
+++ b/data/rules/riskClassification.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCCF8939-57F6-462C-B3E1-9321F7143CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EE69FE4-E63D-4326-AFC6-38D36126BE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="154">
   <si>
     <t>Indicator</t>
   </si>
@@ -474,6 +474,18 @@
   </si>
   <si>
     <t>Financial sanctions (asset freeze)</t>
+  </si>
+  <si>
+    <t>FBI-WANTED</t>
+  </si>
+  <si>
+    <t>US federal wanted persons / fugitives</t>
+  </si>
+  <si>
+    <t>Law Enforcement</t>
+  </si>
+  <si>
+    <t>Wanted / Investigation</t>
   </si>
 </sst>
 </file>
@@ -873,14 +885,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="42.6328125" style="9" customWidth="1"/>
     <col min="2" max="2" width="8.7265625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="22.36328125" style="9" customWidth="1"/>
+    <col min="3" max="3" width="32.81640625" style="9" customWidth="1"/>
     <col min="4" max="4" width="16.81640625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="18.36328125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="22.81640625" style="9" customWidth="1"/>
     <col min="6" max="6" width="11.1796875" style="2" customWidth="1"/>
     <col min="7" max="7" width="35" style="8" customWidth="1"/>
   </cols>
@@ -1185,8 +1197,29 @@
         <v>1</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>